<commit_message>
add risk co owner in import excel in
</commit_message>
<xml_diff>
--- a/app/services/Excel/Test_Tempelate_2.xlsx
+++ b/app/services/Excel/Test_Tempelate_2.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>Department</t>
   </si>
@@ -38,13 +38,7 @@
     <t>Risk Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk Description </t>
-  </si>
-  <si>
     <t>Risk Treatment</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Description</t>
   </si>
   <si>
     <t xml:space="preserve">Inherent Risk Level (Impact/ Likelihood) </t>
@@ -69,9 +63,6 @@
     <t>FIN</t>
   </si>
   <si>
-    <t>Incorrect Assumptions/ Forecasts (RC) for Annual Budget &amp; Plan (RE) resulting inappropriate planning (C )</t>
-  </si>
-  <si>
     <t>3D</t>
   </si>
   <si>
@@ -95,9 +86,6 @@
   </si>
   <si>
     <t>HR</t>
-  </si>
-  <si>
-    <t>Risk of overcompensation or undercompensation and percevied inequity</t>
   </si>
   <si>
     <t>1. Periodic benchmark of compensation against industry standards to remain competitive and retain talent
@@ -107,12 +95,6 @@
 5. Increment review by Brookfield, exceptions are routed through renumeration committee</t>
   </si>
   <si>
-    <t>raj</t>
-  </si>
-  <si>
-    <t>Shiv</t>
-  </si>
-  <si>
     <t>functional_head</t>
   </si>
   <si>
@@ -125,21 +107,6 @@
     <t>JAYRAJ</t>
   </si>
   <si>
-    <t>TEST 3</t>
-  </si>
-  <si>
-    <t>Test 4</t>
-  </si>
-  <si>
-    <t>test 3</t>
-  </si>
-  <si>
-    <t>plan 4</t>
-  </si>
-  <si>
-    <t>Tax compliances including annual returns</t>
-  </si>
-  <si>
     <t>5B</t>
   </si>
   <si>
@@ -149,7 +116,37 @@
     <t>1D</t>
   </si>
   <si>
-    <t>Test 5</t>
+    <t>Risk Co Owner</t>
+  </si>
+  <si>
+    <t>related@example.com</t>
+  </si>
+  <si>
+    <t>TEST 1</t>
+  </si>
+  <si>
+    <t>Test 2</t>
+  </si>
+  <si>
+    <t>Test 3</t>
+  </si>
+  <si>
+    <t>jay@gmail.com</t>
+  </si>
+  <si>
+    <t>aditya@example.com</t>
+  </si>
+  <si>
+    <t>shiv@example.com</t>
+  </si>
+  <si>
+    <t>priya@example.com</t>
+  </si>
+  <si>
+    <t>plan 2</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
 </sst>
 </file>
@@ -229,7 +226,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,12 +265,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -285,7 +276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -308,61 +299,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -374,9 +310,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -403,10 +336,6 @@
     </xf>
     <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -417,32 +346,37 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -732,8 +666,8 @@
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" customWidth="1"/>
     <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="42.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -745,7 +679,7 @@
     <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" s="21" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -758,170 +692,175 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
-    <row r="2" spans="1:14" ht="69" customHeight="1">
-      <c r="A2" s="2"/>
+    <row r="2" spans="1:14" s="21" customFormat="1" ht="69" customHeight="1">
+      <c r="A2" s="22"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="21" customFormat="1" ht="174" customHeight="1">
+      <c r="A3" s="22" t="s">
         <v>11</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="174" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="10">
+        <v>46444</v>
+      </c>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+    </row>
+    <row r="4" spans="1:14" s="21" customFormat="1" ht="144">
+      <c r="A4" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="11">
+        <v>2</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D4" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="25">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" s="21" customFormat="1" ht="60">
+      <c r="A5" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="9">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" s="11">
-        <v>46444</v>
-      </c>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-    </row>
-    <row r="4" spans="1:14" ht="144">
-      <c r="A4" s="13" t="s">
+      <c r="G5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="9"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="14">
-        <v>2</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="17" t="s">
+      <c r="N5" s="22" t="s">
         <v>23</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="20">
-        <v>46264</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="60">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="10">
-        <v>14</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="10"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1"/>
+    <hyperlink ref="D4" r:id="rId2"/>
+    <hyperlink ref="D5" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
+    <hyperlink ref="E3" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>